<commit_message>
Update training venues list to 12 hospitals
</commit_message>
<xml_diff>
--- a/แหล่งฝึก.xlsx
+++ b/แหล่งฝึก.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\งานเบ้บๆ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BAC23FCB-4A18-4E12-B5EF-B6F45D930E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E0AEDA8-55F7-4EFB-8793-5B0C4765F11D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{034C541E-3193-458A-B6A1-F808776ADCE1}"/>
   </bookViews>
@@ -39,15 +39,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>โรงพยาบาลสรรพสิทธิประสงค์</t>
-  </si>
-  <si>
-    <t>องค์การบริหารส่วนจังหวัดอุบลราชธานี</t>
-  </si>
-  <si>
-    <t>องค์การบริหารส่วนจังหวัดศรีสะเกษ</t>
   </si>
   <si>
     <t>โรงพยาบาลศรีสะเกษ</t>
@@ -462,7 +456,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{886E5833-E20D-4DF4-A713-D0D1473387E2}">
-  <dimension ref="D7:D20"/>
+  <dimension ref="D7:D18"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="31.875" bestFit="1" customWidth="1"/>
@@ -528,16 +522,6 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D19" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="20" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D20" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>